<commit_message>
Sprint 2 concluída — Classificação supervisionada de regimes operacionais
Notebooks:
- S2a: Comparação regimes vs dureza SAG (ARI=0,048 → regimes transcendem dureza)
- S2b: Feature engineering (105 features) + split temporal (70/15/15%)
- S2c: Treinamento RF/XGBoost/LightGBM — LightGBM selecionado
  (F1-weighted=0,9704 val | 0,9861 teste | accuracy 98,5%)
- Análise SHAP: top features = vazão espessador, ouvido eletrônico, balança retomada

Artefatos:
- Relatório v4 com métricas, figuras e tabelas atualizadas
- 21 figuras da Sprint 2 (carimbamento, split, confusion matrices, SHAP)
- sql/002_comentarios.sql: documentação completa do PostgreSQL (72/73 tabelas)
- Cronograma atualizado

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Relatorio_Projeto/Cronograma_Acoes_Planejadas.xlsx
+++ b/Relatorio_Projeto/Cronograma_Acoes_Planejadas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScriptsDatamindsPIP\4-Projeto aplicado\Relatorio_Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AFE2975-B812-42B5-9CAD-FCEF3B9F5F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F273C4E4-B2AC-4D4F-9FC7-46FACA96534B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cronograma" sheetId="1" r:id="rId1"/>
@@ -492,6 +492,16 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -511,21 +521,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -833,76 +833,76 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="14" width="7.26953125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="14" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-    </row>
-    <row r="2" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="24" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+    </row>
+    <row r="2" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-    </row>
-    <row r="4" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+    </row>
+    <row r="4" spans="1:15" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11"/>
       <c r="B4" s="11"/>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="23" t="s">
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="16" t="s">
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="18"/>
-      <c r="O4" s="29" t="s">
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="18" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -945,10 +945,10 @@
       <c r="N5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O5" s="30"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A6" s="26" t="s">
+      <c r="O5" s="19"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="29" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -972,8 +972,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A7" s="20"/>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="24"/>
       <c r="B7" s="5" t="s">
         <v>24</v>
       </c>
@@ -997,8 +997,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A8" s="20"/>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="24"/>
       <c r="B8" s="5" t="s">
         <v>25</v>
       </c>
@@ -1022,8 +1022,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A9" s="20"/>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="24"/>
       <c r="B9" s="5" t="s">
         <v>26</v>
       </c>
@@ -1045,8 +1045,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A10" s="20"/>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="24"/>
       <c r="B10" s="5" t="s">
         <v>27</v>
       </c>
@@ -1070,8 +1070,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A11" s="20"/>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="24"/>
       <c r="B11" s="5" t="s">
         <v>28</v>
       </c>
@@ -1093,8 +1093,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A12" s="21"/>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="25"/>
       <c r="B12" s="5" t="s">
         <v>29</v>
       </c>
@@ -1116,8 +1116,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A13" s="27" t="s">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="30" t="s">
         <v>31</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -1137,12 +1137,12 @@
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
-      <c r="O13" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A14" s="20"/>
+      <c r="O13" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="24"/>
       <c r="B14" s="5" t="s">
         <v>33</v>
       </c>
@@ -1160,12 +1160,12 @@
       <c r="L14" s="7"/>
       <c r="M14" s="7"/>
       <c r="N14" s="7"/>
-      <c r="O14" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A15" s="20"/>
+      <c r="O14" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="24"/>
       <c r="B15" s="5" t="s">
         <v>34</v>
       </c>
@@ -1185,12 +1185,12 @@
       <c r="L15" s="7"/>
       <c r="M15" s="7"/>
       <c r="N15" s="7"/>
-      <c r="O15" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A16" s="20"/>
+      <c r="O15" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="24"/>
       <c r="B16" s="5" t="s">
         <v>35</v>
       </c>
@@ -1208,12 +1208,12 @@
       <c r="L16" s="7"/>
       <c r="M16" s="7"/>
       <c r="N16" s="7"/>
-      <c r="O16" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A17" s="20"/>
+      <c r="O16" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="24"/>
       <c r="B17" s="5" t="s">
         <v>36</v>
       </c>
@@ -1233,12 +1233,12 @@
       <c r="L17" s="7"/>
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
-      <c r="O17" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A18" s="20"/>
+      <c r="O17" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="24"/>
       <c r="B18" s="5" t="s">
         <v>37</v>
       </c>
@@ -1256,12 +1256,12 @@
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
-      <c r="O18" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A19" s="20"/>
+      <c r="O18" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="24"/>
       <c r="B19" s="5" t="s">
         <v>38</v>
       </c>
@@ -1281,12 +1281,12 @@
       <c r="L19" s="7"/>
       <c r="M19" s="7"/>
       <c r="N19" s="7"/>
-      <c r="O19" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A20" s="21"/>
+      <c r="O19" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="25"/>
       <c r="B20" s="5" t="s">
         <v>39</v>
       </c>
@@ -1304,12 +1304,12 @@
       <c r="L20" s="7"/>
       <c r="M20" s="7"/>
       <c r="N20" s="7"/>
-      <c r="O20" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A21" s="19" t="s">
+      <c r="O20" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="23" t="s">
         <v>40</v>
       </c>
       <c r="B21" s="5" t="s">
@@ -1333,8 +1333,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A22" s="20"/>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="24"/>
       <c r="B22" s="5" t="s">
         <v>42</v>
       </c>
@@ -1358,8 +1358,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A23" s="20"/>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="24"/>
       <c r="B23" s="5" t="s">
         <v>43</v>
       </c>
@@ -1381,8 +1381,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A24" s="20"/>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="24"/>
       <c r="B24" s="5" t="s">
         <v>44</v>
       </c>
@@ -1406,8 +1406,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A25" s="20"/>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="24"/>
       <c r="B25" s="5" t="s">
         <v>45</v>
       </c>
@@ -1429,8 +1429,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A26" s="21"/>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="25"/>
       <c r="B26" s="5" t="s">
         <v>46</v>
       </c>
@@ -1454,17 +1454,17 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
         <v>30</v>
       </c>

</xml_diff>